<commit_message>
Update Login Test page
</commit_message>
<xml_diff>
--- a/src/test/resources/testData.xlsx
+++ b/src/test/resources/testData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sumreen\IdeaProjects\saucedemo-selenium-java-framework\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C997EAB-A475-4C22-BFB4-B6166D952738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EE6EEA3-1FF6-429F-AFDE-963878ACF133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{54D39150-26B2-44CE-95A6-9D876FBA1E81}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
   <si>
     <t>Username</t>
   </si>
@@ -64,6 +64,15 @@
   </si>
   <si>
     <t>Epic sadface: Sorry, this user has been locked out.</t>
+  </si>
+  <si>
+    <t>Epic sadface: Username and password do not match any user in this service</t>
+  </si>
+  <si>
+    <t>hghghmgjmhjmhj,ghmfggcg</t>
+  </si>
+  <si>
+    <t>invalid</t>
   </si>
 </sst>
 </file>
@@ -474,7 +483,7 @@
       <c r="C2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="4" t="s">
         <v>7</v>
       </c>
     </row>
@@ -506,9 +515,19 @@
         <v>404</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
+    <row r="5" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B6" s="2"/>

</xml_diff>